<commit_message>
Update Gold Master and xlsm files
</commit_message>
<xml_diff>
--- a/doctool/test/auto/scenario12/システム機能設計書_サンプル_S12_expected.xlsx
+++ b/doctool/test/auto/scenario12/システム機能設計書_サンプル_S12_expected.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PJ\01.Nablarch\repo\review-support-tool\doctool\test\temp_dir\scenario11\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PJ\01.Nablarch\repo\review-support-tool\doctool\test\temp_dir\scenario12\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86FD71B9-0911-44C0-B56F-BEB4FBFF613C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B620656B-FBA0-40E1-98BE-E0B9F421FE82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="38700" windowHeight="15345" tabRatio="822" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4290" yWindow="4290" windowWidth="38700" windowHeight="15345" tabRatio="822" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="レビュー結果1回目" sheetId="9" r:id="rId1"/>
@@ -1112,30 +1112,39 @@
   </si>
   <si>
     <t>01_要件漏れ</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>02_要件誤り</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>11_機能・仕様漏れ</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>12_機能・仕様誤り</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>21_設計・ドキュメント規約違反</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>22_記述誤り</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>91_疑問点、確認</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>92_改善要望</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>93_仕様変更</t>
+    <phoneticPr fontId="13"/>
   </si>
   <si>
     <t>計</t>
@@ -1220,7 +1229,7 @@
     <t>D00001</t>
   </si>
   <si>
-    <t>システム機能設計書_サンプル_S11</t>
+    <t>システム機能設計書_サンプル_S12</t>
   </si>
   <si>
     <t>B5</t>
@@ -2689,7 +2698,7 @@
     <xf numFmtId="0" fontId="26" fillId="8" borderId="10" xfId="11" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="11" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="178" fontId="14" fillId="0" borderId="10" xfId="11" applyNumberFormat="1" applyBorder="1">
@@ -3182,7 +3191,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8CC69391-7C2B-434F-852D-1D6B4A897CB7}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34C990A3-66C8-4B83-B752-AC753CA0B271}">
   <sheetPr codeName="SheetTemplate">
     <tabColor indexed="44"/>
     <pageSetUpPr fitToPage="1"/>
@@ -3850,20 +3859,20 @@
     <mergeCell ref="E18:J18"/>
   </mergeCells>
   <phoneticPr fontId="10"/>
-  <conditionalFormatting sqref="A15:T18">
+  <conditionalFormatting sqref="A15:K18">
     <cfRule type="expression" dxfId="0" priority="1" stopIfTrue="1">
       <formula>$K15="済"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K15:K18" xr:uid="{09B388DD-82B6-4FD2-B563-0F95E518028F}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K15:K18" xr:uid="{45549F93-8136-4A85-A7CC-B3B7B43851E1}">
       <formula1>"未,済"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="B15" location="'2. WA1020101(プロジェクト登録画面)'!$B$5" display="'2. WA1020101(プロジェクト登録画面)'!$B$5" xr:uid="{9946AF56-77B1-47FF-B88E-75AC1DFC688E}"/>
-    <hyperlink ref="B16" location="'2. WA1020101(プロジェクト登録画面)'!$E$60" display="'2. WA1020101(プロジェクト登録画面)'!$E$60" xr:uid="{4BBE0EC0-1D9E-4484-815C-EBD337BDDE25}"/>
-    <hyperlink ref="B17" location="'2. WA1020101(プロジェクト登録画面)'!$E$62" display="'2. WA1020101(プロジェクト登録画面)'!$E$62" xr:uid="{7A636145-8E3F-4204-AA25-D3881FB018C9}"/>
+    <hyperlink ref="B15" location="'2. WA1020101(プロジェクト登録画面)'!$B$5" display="'2. WA1020101(プロジェクト登録画面)'!$B$5" xr:uid="{DD202A32-84C4-43D7-92DD-88609BDE0C65}"/>
+    <hyperlink ref="B16" location="'2. WA1020101(プロジェクト登録画面)'!$E$60" display="'2. WA1020101(プロジェクト登録画面)'!$E$60" xr:uid="{7CC6AA68-2686-42BE-89BC-E7CD7022CBB6}"/>
+    <hyperlink ref="B17" location="'2. WA1020101(プロジェクト登録画面)'!$E$62" display="'2. WA1020101(プロジェクト登録画面)'!$E$62" xr:uid="{803B4D61-B0D7-4C7D-A3FF-33CEECE1FD17}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51200000000000001" footer="0.51200000000000001"/>
   <pageSetup paperSize="9" scale="86" orientation="landscape" verticalDpi="200" r:id="rId1"/>

</xml_diff>